<commit_message>
PhotosyntheticPathway added to harmonized trait definition
</commit_message>
<xml_diff>
--- a/data-raw/HarmonizedTraitDefinition.xlsx
+++ b/data-raw/HarmonizedTraitDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="224">
   <si>
     <t xml:space="preserve">Definition</t>
   </si>
@@ -131,6 +131,15 @@
   </si>
   <si>
     <t xml:space="preserve">light-demanding,shade-tolerant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Photosynthetic pathway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PhotosyntheticPathway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C3,C4,CAM</t>
   </si>
   <si>
     <t xml:space="preserve">Duration of leaves (leaf lifespan)</t>
@@ -973,7 +982,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1031"/>
+  <dimension ref="A1:H1032"/>
   <sheetFormatPr defaultColWidth="12.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="111.7"/>
@@ -1188,13 +1197,13 @@
         <v>38</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
@@ -1213,9 +1222,7 @@
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1229,7 +1236,7 @@
         <v>20</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -1240,16 +1247,16 @@
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -1260,16 +1267,16 @@
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -1288,49 +1295,47 @@
       <c r="C16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>52</v>
+      </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>55</v>
-      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3" t="n">
@@ -1340,36 +1345,38 @@
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>20</v>
+      <c r="E19" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
+      <c r="G19" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E20" s="3"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1382,32 +1389,35 @@
       <c r="C21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="1" t="s">
-        <v>69</v>
-      </c>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
       <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
+      <c r="G22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
@@ -1419,33 +1429,28 @@
       <c r="C23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="F23" s="3"/>
-      <c r="G23" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G23" s="3"/>
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="C24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>72</v>
-      </c>
       <c r="E24" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3" t="n">
@@ -1455,19 +1460,19 @@
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3" t="n">
@@ -1477,18 +1482,20 @@
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" s="3"/>
+        <v>75</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3" t="n">
         <v>0</v>
@@ -1497,18 +1504,18 @@
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E27" s="5"/>
+      <c r="D27" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3" t="n">
         <v>0</v>
@@ -1526,7 +1533,7 @@
         <v>20</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E28" s="5"/>
       <c r="F28" s="3"/>
@@ -1537,16 +1544,16 @@
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>82</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="3"/>
@@ -1557,20 +1564,22 @@
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="E30" s="3"/>
+      <c r="D30" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E30" s="5"/>
       <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
+      <c r="G30" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1584,26 +1593,26 @@
         <v>20</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>89</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B32" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
@@ -1619,7 +1628,7 @@
         <v>20</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
@@ -1628,16 +1637,16 @@
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -1646,15 +1655,17 @@
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D35" s="3"/>
+      <c r="D35" s="3" t="s">
+        <v>92</v>
+      </c>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -1662,36 +1673,32 @@
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D36" s="3" t="s">
-        <v>89</v>
-      </c>
+      <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
-      <c r="H36" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -1702,16 +1709,16 @@
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -1722,16 +1729,16 @@
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -1742,16 +1749,16 @@
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -1762,22 +1769,23 @@
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>109</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="E41" s="3"/>
       <c r="F41" s="3"/>
-      <c r="G41" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
@@ -1790,7 +1798,7 @@
         <v>20</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3" t="n">
@@ -1800,18 +1808,17 @@
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D43" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B43" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E43" s="3"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3" t="n">
         <v>0</v>
@@ -1829,7 +1836,7 @@
         <v>20</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
@@ -1840,16 +1847,16 @@
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>114</v>
       </c>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
@@ -1860,16 +1867,16 @@
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
@@ -1929,7 +1936,7 @@
         <v>20</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
@@ -1940,36 +1947,36 @@
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D50" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="3"/>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -1980,16 +1987,16 @@
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
@@ -2000,54 +2007,54 @@
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D53" s="3"/>
+      <c r="D53" s="3" t="s">
+        <v>92</v>
+      </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
-      <c r="G53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D54" s="3" t="s">
-        <v>89</v>
-      </c>
+      <c r="D54" s="3"/>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
@@ -2058,16 +2065,16 @@
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
@@ -2078,54 +2085,54 @@
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D57" s="3"/>
+      <c r="D57" s="3" t="s">
+        <v>92</v>
+      </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
-      <c r="G57" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D58" s="3" t="s">
-        <v>89</v>
-      </c>
+      <c r="D58" s="3"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="3"/>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
@@ -2136,16 +2143,16 @@
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
@@ -2156,35 +2163,35 @@
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D61" s="3"/>
+      <c r="D61" s="3" t="s">
+        <v>92</v>
+      </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
-      <c r="G61" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="H61" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>114</v>
-      </c>
+      <c r="D62" s="3"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
       <c r="G62" s="3" t="n">
@@ -2194,16 +2201,16 @@
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
@@ -2222,31 +2229,31 @@
       <c r="C64" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D64" s="5"/>
-      <c r="E64" s="5"/>
+      <c r="D64" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E64" s="3"/>
       <c r="F64" s="3"/>
       <c r="G64" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H64" s="3"/>
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D65" s="5" t="s">
-        <v>154</v>
-      </c>
+      <c r="D65" s="5"/>
       <c r="E65" s="5"/>
       <c r="F65" s="3"/>
       <c r="G65" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H65" s="3"/>
     </row>
@@ -2280,50 +2287,50 @@
       <c r="C67" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D67" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="E67" s="3"/>
+      <c r="D67" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="E67" s="5"/>
       <c r="F67" s="3"/>
       <c r="G67" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H67" s="3" t="n">
-        <v>100</v>
-      </c>
+      <c r="H67" s="3"/>
     </row>
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>49</v>
+        <v>152</v>
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3"/>
       <c r="G68" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H68" s="3"/>
+      <c r="H68" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
@@ -2334,10 +2341,10 @@
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>20</v>
@@ -2354,16 +2361,16 @@
     </row>
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3"/>
@@ -2374,16 +2381,16 @@
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>170</v>
+        <v>45</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
@@ -2423,7 +2430,7 @@
         <v>20</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>58</v>
+        <v>176</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
@@ -2434,16 +2441,16 @@
     </row>
     <row r="75" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C75" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>178</v>
+        <v>61</v>
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
@@ -2462,18 +2469,22 @@
       <c r="C76" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D76" s="3"/>
+      <c r="D76" s="3" t="s">
+        <v>181</v>
+      </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
-      <c r="G76" s="3"/>
+      <c r="G76" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H76" s="3"/>
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>20</v>
@@ -2486,17 +2497,15 @@
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D78" s="3" t="s">
-        <v>185</v>
-      </c>
+      <c r="D78" s="3"/>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -2517,9 +2526,7 @@
       </c>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
-      <c r="G79" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G79" s="3"/>
       <c r="H79" s="3"/>
     </row>
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2533,7 +2540,7 @@
         <v>20</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
@@ -2544,16 +2551,16 @@
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D81" s="3" t="s">
         <v>191</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="C81" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>188</v>
       </c>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
@@ -2564,16 +2571,16 @@
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>69</v>
+        <v>191</v>
       </c>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
@@ -2584,16 +2591,16 @@
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
@@ -2604,16 +2611,16 @@
     </row>
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C84" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
@@ -2624,20 +2631,22 @@
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>201</v>
+        <v>72</v>
       </c>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
-      <c r="G85" s="3"/>
+      <c r="G85" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H85" s="3"/>
     </row>
     <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2651,7 +2660,7 @@
         <v>20</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
@@ -2660,16 +2669,16 @@
     </row>
     <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C87" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
@@ -2678,16 +2687,16 @@
     </row>
     <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
@@ -2696,16 +2705,16 @@
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
@@ -2723,7 +2732,7 @@
         <v>20</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>185</v>
+        <v>213</v>
       </c>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
@@ -2732,40 +2741,36 @@
     </row>
     <row r="91" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D91" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>188</v>
+      </c>
       <c r="E91" s="3"/>
-      <c r="F91" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="G91" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H91" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="H91" s="3"/>
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B92" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="B92" s="3" t="s">
+      <c r="C92" s="3" t="s">
         <v>218</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>215</v>
       </c>
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="G92" s="3" t="n">
         <v>0</v>
@@ -2776,25 +2781,46 @@
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>20</v>
+        <v>218</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
-      <c r="F93" s="3"/>
+      <c r="F93" s="3" t="s">
+        <v>219</v>
+      </c>
       <c r="G93" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H93" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A94" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="3" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3732,6 +3758,7 @@
     <row r="1029" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1030" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1031" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1032" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>

</xml_diff>

<commit_message>
update harmonized trait definition
</commit_message>
<xml_diff>
--- a/data-raw/HarmonizedTraitDefinition.xlsx
+++ b/data-raw/HarmonizedTraitDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="227">
   <si>
     <t xml:space="preserve">Definition</t>
   </si>
@@ -140,6 +140,15 @@
   </si>
   <si>
     <t xml:space="preserve">C3,C4,CAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wood porosity type (for woody angiosperms)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WoodPorosityType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ring-porous,semi-ring-porous,diffuse-porous</t>
   </si>
   <si>
     <t xml:space="preserve">Duration of leaves (leaf lifespan)</t>
@@ -436,7 +445,7 @@
     <t xml:space="preserve">10-4 kg m-1 MPa-1 s-1</t>
   </si>
   <si>
-    <t xml:space="preserve">Maximum leaf hydraulic conductance</t>
+    <t xml:space="preserve">Maximum leaf hydraulic conductance (per leaf area)</t>
   </si>
   <si>
     <t xml:space="preserve">kleaf</t>
@@ -445,7 +454,7 @@
     <t xml:space="preserve">mmol m-2 s-1 MPa-1</t>
   </si>
   <si>
-    <t xml:space="preserve">Maximum whole-plant hydraulic conductance</t>
+    <t xml:space="preserve">Maximum whole-plant hydraulic conductance (per leaf area)</t>
   </si>
   <si>
     <t xml:space="preserve">kplant</t>
@@ -982,7 +991,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H1032"/>
+  <dimension ref="A1:H1033"/>
   <sheetFormatPr defaultColWidth="12.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="111.7"/>
@@ -1215,13 +1224,13 @@
         <v>41</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
@@ -1240,9 +1249,7 @@
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1256,7 +1263,7 @@
         <v>20</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -1267,16 +1274,16 @@
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -1287,16 +1294,16 @@
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -1315,49 +1322,47 @@
       <c r="C17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
+      <c r="G17" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>58</v>
-      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
       <c r="F18" s="3"/>
-      <c r="G18" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3" t="n">
@@ -1367,36 +1372,38 @@
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>20</v>
+      <c r="E20" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
+      <c r="G20" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E21" s="3"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1409,32 +1416,35 @@
       <c r="C22" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="3" t="s">
+        <v>70</v>
+      </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="1" t="s">
-        <v>72</v>
-      </c>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
       <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
+      <c r="G23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
@@ -1446,33 +1456,28 @@
       <c r="C24" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="D24" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>76</v>
-      </c>
       <c r="F24" s="3"/>
-      <c r="G24" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G24" s="3"/>
       <c r="H24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="C25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="E25" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3" t="n">
@@ -1482,19 +1487,19 @@
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3" t="n">
@@ -1504,18 +1509,20 @@
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E27" s="3"/>
+        <v>78</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>79</v>
+      </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3" t="n">
         <v>0</v>
@@ -1524,18 +1531,18 @@
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E28" s="5"/>
+      <c r="D28" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3" t="n">
         <v>0</v>
@@ -1553,7 +1560,7 @@
         <v>20</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" s="3"/>
@@ -1564,16 +1571,16 @@
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="E30" s="5"/>
       <c r="F30" s="3"/>
@@ -1584,20 +1591,22 @@
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E31" s="3"/>
+      <c r="D31" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E31" s="5"/>
       <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
+      <c r="G31" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1611,26 +1620,26 @@
         <v>20</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>92</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B33" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
@@ -1646,7 +1655,7 @@
         <v>20</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -1655,16 +1664,16 @@
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
@@ -1673,15 +1682,17 @@
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D36" s="3"/>
+      <c r="D36" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -1689,36 +1700,32 @@
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>92</v>
-      </c>
+      <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
-      <c r="H37" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="H37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -1729,16 +1736,16 @@
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -1749,16 +1756,16 @@
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -1769,16 +1776,16 @@
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -1789,22 +1796,23 @@
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>112</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="E42" s="3"/>
       <c r="F42" s="3"/>
-      <c r="G42" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
@@ -1817,7 +1825,7 @@
         <v>20</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3" t="n">
@@ -1827,18 +1835,17 @@
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E44" s="3"/>
       <c r="F44" s="3"/>
       <c r="G44" s="3" t="n">
         <v>0</v>
@@ -1856,7 +1863,7 @@
         <v>20</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
@@ -1867,16 +1874,16 @@
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
@@ -1887,16 +1894,16 @@
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
@@ -1956,7 +1963,7 @@
         <v>20</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -1967,36 +1974,36 @@
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D51" s="3" t="s">
         <v>133</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>92</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="3"/>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
@@ -2007,16 +2014,16 @@
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -2027,54 +2034,54 @@
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D54" s="3"/>
+      <c r="D54" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
-      <c r="G54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>92</v>
-      </c>
+      <c r="D55" s="3"/>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
-      <c r="G55" s="3"/>
-      <c r="H55" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="3"/>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
@@ -2085,16 +2092,16 @@
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
@@ -2105,54 +2112,54 @@
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D58" s="3"/>
+      <c r="D58" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
-      <c r="G58" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="H58" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D59" s="3" t="s">
-        <v>92</v>
-      </c>
+      <c r="D59" s="3"/>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
-      <c r="G59" s="3"/>
-      <c r="H59" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" s="3"/>
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
@@ -2163,16 +2170,16 @@
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
@@ -2183,35 +2190,35 @@
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D62" s="3"/>
+      <c r="D62" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="E62" s="3"/>
       <c r="F62" s="3"/>
-      <c r="G62" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D63" s="3" t="s">
-        <v>117</v>
-      </c>
+      <c r="D63" s="3"/>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
       <c r="G63" s="3" t="n">
@@ -2221,16 +2228,16 @@
     </row>
     <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C64" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>152</v>
+        <v>120</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
@@ -2249,31 +2256,31 @@
       <c r="C65" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D65" s="5"/>
-      <c r="E65" s="5"/>
+      <c r="D65" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E65" s="3"/>
       <c r="F65" s="3"/>
       <c r="G65" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H65" s="3"/>
     </row>
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C66" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D66" s="5" t="s">
-        <v>157</v>
-      </c>
+      <c r="D66" s="5"/>
       <c r="E66" s="5"/>
       <c r="F66" s="3"/>
       <c r="G66" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H66" s="3"/>
     </row>
@@ -2307,50 +2314,50 @@
       <c r="C68" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D68" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="E68" s="3"/>
+      <c r="D68" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="E68" s="5"/>
       <c r="F68" s="3"/>
       <c r="G68" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H68" s="3" t="n">
-        <v>100</v>
-      </c>
+      <c r="H68" s="3"/>
     </row>
     <row r="69" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C69" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>52</v>
+        <v>155</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
       <c r="G69" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H69" s="3"/>
+      <c r="H69" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
@@ -2361,10 +2368,10 @@
     </row>
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>20</v>
@@ -2381,16 +2388,16 @@
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
@@ -2401,16 +2408,16 @@
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>173</v>
+        <v>48</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
@@ -2450,7 +2457,7 @@
         <v>20</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>61</v>
+        <v>179</v>
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
@@ -2461,16 +2468,16 @@
     </row>
     <row r="76" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>181</v>
+        <v>64</v>
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
@@ -2489,18 +2496,22 @@
       <c r="C77" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D77" s="3"/>
+      <c r="D77" s="3" t="s">
+        <v>184</v>
+      </c>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
-      <c r="G77" s="3"/>
+      <c r="G77" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H77" s="3"/>
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>20</v>
@@ -2513,17 +2524,15 @@
     </row>
     <row r="79" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C79" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D79" s="3" t="s">
-        <v>188</v>
-      </c>
+      <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -2544,9 +2553,7 @@
       </c>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
-      <c r="G80" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="G80" s="3"/>
       <c r="H80" s="3"/>
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2560,7 +2567,7 @@
         <v>20</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="E81" s="3"/>
       <c r="F81" s="3"/>
@@ -2571,16 +2578,16 @@
     </row>
     <row r="82" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D82" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="B82" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="C82" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D82" s="3" t="s">
-        <v>191</v>
       </c>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
@@ -2591,16 +2598,16 @@
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>72</v>
+        <v>194</v>
       </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
@@ -2611,16 +2618,16 @@
     </row>
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C84" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
@@ -2631,16 +2638,16 @@
     </row>
     <row r="85" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
@@ -2651,20 +2658,22 @@
     </row>
     <row r="86" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>204</v>
+        <v>75</v>
       </c>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
+      <c r="G86" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="H86" s="3"/>
     </row>
     <row r="87" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2678,7 +2687,7 @@
         <v>20</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>188</v>
+        <v>207</v>
       </c>
       <c r="E87" s="3"/>
       <c r="F87" s="3"/>
@@ -2687,16 +2696,16 @@
     </row>
     <row r="88" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
@@ -2705,16 +2714,16 @@
     </row>
     <row r="89" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
@@ -2723,16 +2732,16 @@
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C90" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
@@ -2750,7 +2759,7 @@
         <v>20</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
@@ -2759,40 +2768,36 @@
     </row>
     <row r="92" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="D92" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>191</v>
+      </c>
       <c r="E92" s="3"/>
-      <c r="F92" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="G92" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H92" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
     </row>
     <row r="93" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B93" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B93" s="3" t="s">
+      <c r="C93" s="3" t="s">
         <v>221</v>
-      </c>
-      <c r="C93" s="3" t="s">
-        <v>218</v>
       </c>
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="G93" s="3" t="n">
         <v>0</v>
@@ -2803,25 +2808,46 @@
     </row>
     <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>20</v>
+        <v>221</v>
       </c>
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
-      <c r="F94" s="3"/>
+      <c r="F94" s="3" t="s">
+        <v>222</v>
+      </c>
       <c r="G94" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H94" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A95" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="3" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="97" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3759,6 +3785,7 @@
     <row r="1030" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1031" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1032" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1033" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>

</xml_diff>

<commit_message>
update priority on trait means + spparams rebuild
</commit_message>
<xml_diff>
--- a/data-raw/HarmonizedTraitDefinition.xlsx
+++ b/data-raw/HarmonizedTraitDefinition.xlsx
@@ -1696,7 +1696,9 @@
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
+      <c r="H36" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">

</xml_diff>

<commit_message>
update trait definition with stomatal conductance
</commit_message>
<xml_diff>
--- a/data-raw/HarmonizedTraitDefinition.xlsx
+++ b/data-raw/HarmonizedTraitDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="240">
   <si>
     <t xml:space="preserve">Definition</t>
   </si>
@@ -304,10 +304,10 @@
     <t xml:space="preserve">mm-2</t>
   </si>
   <si>
-    <t xml:space="preserve">Maximum stomatal conductance to water vapor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gswmax</t>
+    <t xml:space="preserve">Stomatal conductance to water vapor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gsw</t>
   </si>
   <si>
     <r>
@@ -341,6 +341,12 @@
       </rPr>
       <t xml:space="preserve">m-2</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum stomatal conductance to water vapor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gswmax</t>
   </si>
   <si>
     <t xml:space="preserve">Minimum stomatal conductance to water vapor</t>
@@ -1024,7 +1030,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J1035"/>
+  <dimension ref="A1:J1036"/>
   <sheetFormatPr defaultColWidth="12.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="111.7"/>
@@ -1696,9 +1702,9 @@
       <c r="D31" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3" t="n">
         <v>0</v>
@@ -1759,33 +1765,34 @@
       <c r="C34" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="G34" s="3"/>
+      <c r="D34" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
       <c r="H34" s="3"/>
-      <c r="I34" s="3"/>
+      <c r="I34" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="E35" s="3"/>
+      <c r="F35" s="3" t="s">
         <v>106</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
@@ -1803,10 +1810,11 @@
         <v>22</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
+        <v>105</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>106</v>
+      </c>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
@@ -1814,16 +1822,16 @@
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="C37" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>103</v>
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -1843,18 +1851,14 @@
         <v>22</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E38" s="3"/>
-      <c r="F38" s="3" t="s">
-        <v>104</v>
-      </c>
+      <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
-      <c r="J38" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="J38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
@@ -1866,13 +1870,19 @@
       <c r="C39" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D39" s="3"/>
+      <c r="D39" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
+      <c r="F39" s="3" t="s">
+        <v>106</v>
+      </c>
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
-      <c r="J39" s="3"/>
+      <c r="J39" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
@@ -1884,30 +1894,26 @@
       <c r="C40" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D40" s="3" t="s">
-        <v>103</v>
-      </c>
+      <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
-      <c r="J40" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="J40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C41" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -1920,16 +1926,16 @@
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
@@ -1942,16 +1948,16 @@
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -1964,16 +1970,16 @@
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
@@ -1986,7 +1992,7 @@
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>123</v>
@@ -1995,26 +2001,29 @@
         <v>22</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>124</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
       <c r="H45" s="3"/>
-      <c r="I45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="C46" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D46" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="H46" s="3"/>
       <c r="I46" s="3" t="n">
@@ -2033,11 +2042,8 @@
         <v>22</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
+        <v>126</v>
+      </c>
       <c r="H47" s="3"/>
       <c r="I47" s="3" t="n">
         <v>0</v>
@@ -2046,16 +2052,16 @@
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="C48" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D48" s="3" t="s">
         <v>131</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
@@ -2077,7 +2083,7 @@
         <v>22</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
@@ -2099,7 +2105,7 @@
         <v>22</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -2112,16 +2118,16 @@
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B51" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="B51" s="3" t="s">
+      <c r="C51" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D51" s="3" t="s">
         <v>138</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>139</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -2134,16 +2140,16 @@
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B52" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="C52" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D52" s="3" t="s">
         <v>141</v>
-      </c>
-      <c r="C52" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>142</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
@@ -2156,16 +2162,16 @@
     </row>
     <row r="53" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="C53" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D53" s="3" t="s">
         <v>144</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>142</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -2187,40 +2193,36 @@
         <v>22</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>103</v>
+        <v>144</v>
       </c>
       <c r="E54" s="3"/>
-      <c r="F54" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>148</v>
-      </c>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
       <c r="H54" s="3"/>
-      <c r="I54" s="3"/>
-      <c r="J54" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="I54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="3"/>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H55" s="3"/>
       <c r="I55" s="3"/>
@@ -2230,23 +2232,23 @@
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C56" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H56" s="3"/>
       <c r="I56" s="3"/>
@@ -2256,31 +2258,33 @@
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D57" s="3"/>
+      <c r="D57" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H57" s="3"/>
-      <c r="I57" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>153</v>
@@ -2288,41 +2292,39 @@
       <c r="C58" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D58" s="3" t="s">
-        <v>103</v>
-      </c>
+      <c r="D58" s="3"/>
       <c r="E58" s="3"/>
       <c r="F58" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H58" s="3"/>
-      <c r="I58" s="3"/>
-      <c r="J58" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="I58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="3"/>
     </row>
     <row r="59" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C59" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H59" s="3"/>
       <c r="I59" s="3"/>
@@ -2332,23 +2334,23 @@
     </row>
     <row r="60" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H60" s="3"/>
       <c r="I60" s="3"/>
@@ -2358,31 +2360,33 @@
     </row>
     <row r="61" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D61" s="3"/>
+      <c r="D61" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H61" s="3"/>
-      <c r="I61" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" s="3"/>
+      <c r="I61" s="3"/>
+      <c r="J61" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>158</v>
@@ -2390,41 +2394,39 @@
       <c r="C62" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>103</v>
-      </c>
+      <c r="D62" s="3"/>
       <c r="E62" s="3"/>
       <c r="F62" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H62" s="3"/>
-      <c r="I62" s="3"/>
-      <c r="J62" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="I62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="3"/>
     </row>
     <row r="63" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H63" s="3"/>
       <c r="I63" s="3"/>
@@ -2434,23 +2436,23 @@
     </row>
     <row r="64" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C64" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H64" s="3"/>
       <c r="I64" s="3"/>
@@ -2460,31 +2462,33 @@
     </row>
     <row r="65" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D65" s="3"/>
+      <c r="D65" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="E65" s="3"/>
       <c r="F65" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H65" s="3"/>
-      <c r="I65" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" s="3"/>
+      <c r="I65" s="3"/>
+      <c r="J65" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>163</v>
@@ -2492,12 +2496,14 @@
       <c r="C66" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D66" s="3" t="s">
-        <v>129</v>
-      </c>
+      <c r="D66" s="3"/>
       <c r="E66" s="3"/>
-      <c r="F66" s="3"/>
-      <c r="G66" s="3"/>
+      <c r="F66" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>150</v>
+      </c>
       <c r="H66" s="3"/>
       <c r="I66" s="3" t="n">
         <v>0</v>
@@ -2515,7 +2521,7 @@
         <v>22</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>166</v>
+        <v>131</v>
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
@@ -2528,21 +2534,23 @@
     </row>
     <row r="68" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B68" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B68" s="3" t="s">
+      <c r="C68" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D68" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="C68" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D68" s="5"/>
-      <c r="E68" s="5"/>
-      <c r="F68" s="5"/>
-      <c r="G68" s="5"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
       <c r="H68" s="3"/>
       <c r="I68" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J68" s="3"/>
     </row>
@@ -2556,30 +2564,28 @@
       <c r="C69" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D69" s="5" t="s">
-        <v>171</v>
-      </c>
+      <c r="D69" s="5"/>
       <c r="E69" s="5"/>
       <c r="F69" s="5"/>
       <c r="G69" s="5"/>
       <c r="H69" s="3"/>
       <c r="I69" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J69" s="3"/>
     </row>
     <row r="70" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B70" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="C70" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D70" s="5" t="s">
         <v>173</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D70" s="5" t="s">
-        <v>174</v>
       </c>
       <c r="E70" s="5"/>
       <c r="F70" s="5"/>
@@ -2592,27 +2598,25 @@
     </row>
     <row r="71" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B71" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B71" s="3" t="s">
+      <c r="C71" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D71" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="C71" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="E71" s="3"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="3"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
       <c r="H71" s="3"/>
       <c r="I71" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J71" s="3" t="n">
-        <v>100</v>
-      </c>
+      <c r="J71" s="3"/>
     </row>
     <row r="72" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
@@ -2625,7 +2629,7 @@
         <v>22</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>57</v>
+        <v>168</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
@@ -2634,7 +2638,9 @@
       <c r="I72" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J72" s="3"/>
+      <c r="J72" s="3" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
@@ -2647,7 +2653,7 @@
         <v>22</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3"/>
@@ -2669,7 +2675,7 @@
         <v>22</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
@@ -2713,7 +2719,7 @@
         <v>22</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>187</v>
+        <v>50</v>
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
@@ -2726,16 +2732,16 @@
     </row>
     <row r="77" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B77" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="C77" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D77" s="3" t="s">
         <v>189</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>190</v>
       </c>
       <c r="E77" s="3"/>
       <c r="F77" s="3"/>
@@ -2748,16 +2754,16 @@
     </row>
     <row r="78" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B78" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="C78" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D78" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="E78" s="3"/>
       <c r="F78" s="3"/>
@@ -2779,7 +2785,7 @@
         <v>22</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>195</v>
+        <v>66</v>
       </c>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
@@ -2792,20 +2798,24 @@
     </row>
     <row r="80" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B80" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="C80" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D80" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="C80" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
       <c r="G80" s="3"/>
       <c r="H80" s="3"/>
-      <c r="I80" s="3"/>
+      <c r="I80" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J80" s="3"/>
     </row>
     <row r="81" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2836,9 +2846,7 @@
       <c r="C82" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D82" s="3" t="s">
-        <v>202</v>
-      </c>
+      <c r="D82" s="3"/>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
       <c r="G82" s="3"/>
@@ -2848,38 +2856,36 @@
     </row>
     <row r="83" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B83" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="B83" s="3" t="s">
+      <c r="C83" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D83" s="3" t="s">
         <v>204</v>
-      </c>
-      <c r="C83" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D83" s="3" t="s">
-        <v>205</v>
       </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
       <c r="G83" s="3"/>
       <c r="H83" s="3"/>
-      <c r="I83" s="3" t="n">
-        <v>0</v>
-      </c>
+      <c r="I83" s="3"/>
       <c r="J83" s="3"/>
     </row>
     <row r="84" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B84" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="B84" s="3" t="s">
+      <c r="C84" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D84" s="3" t="s">
         <v>207</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>205</v>
       </c>
       <c r="E84" s="3"/>
       <c r="F84" s="3"/>
@@ -2901,7 +2907,7 @@
         <v>22</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E85" s="3"/>
       <c r="F85" s="3"/>
@@ -2923,7 +2929,7 @@
         <v>22</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>77</v>
+        <v>207</v>
       </c>
       <c r="E86" s="3"/>
       <c r="F86" s="3"/>
@@ -2989,27 +2995,29 @@
         <v>22</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>218</v>
+        <v>77</v>
       </c>
       <c r="E89" s="3"/>
       <c r="F89" s="3"/>
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
-      <c r="I89" s="3"/>
+      <c r="I89" s="3" t="n">
+        <v>0</v>
+      </c>
       <c r="J89" s="3"/>
     </row>
     <row r="90" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B90" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="B90" s="3" t="s">
+      <c r="C90" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D90" s="3" t="s">
         <v>220</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>202</v>
       </c>
       <c r="E90" s="3"/>
       <c r="F90" s="3"/>
@@ -3029,7 +3037,7 @@
         <v>22</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E91" s="3"/>
       <c r="F91" s="3"/>
@@ -3049,7 +3057,7 @@
         <v>22</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E92" s="3"/>
       <c r="F92" s="3"/>
@@ -3069,7 +3077,7 @@
         <v>22</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>227</v>
+        <v>204</v>
       </c>
       <c r="E93" s="3"/>
       <c r="F93" s="3"/>
@@ -3080,16 +3088,16 @@
     </row>
     <row r="94" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B94" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="B94" s="3" t="s">
+      <c r="C94" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D94" s="3" t="s">
         <v>229</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>202</v>
       </c>
       <c r="E94" s="3"/>
       <c r="F94" s="3"/>
@@ -3106,38 +3114,34 @@
         <v>231</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="D95" s="3"/>
+        <v>22</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>204</v>
+      </c>
       <c r="E95" s="3"/>
       <c r="F95" s="3"/>
       <c r="G95" s="3"/>
-      <c r="H95" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="I95" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J95" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="H95" s="3"/>
+      <c r="I95" s="3"/>
+      <c r="J95" s="3"/>
     </row>
     <row r="96" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C96" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>232</v>
       </c>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3"/>
       <c r="G96" s="3"/>
       <c r="H96" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I96" s="3" t="n">
         <v>0</v>
@@ -3154,21 +3158,44 @@
         <v>237</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>22</v>
+        <v>234</v>
       </c>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
       <c r="F97" s="3"/>
       <c r="G97" s="3"/>
-      <c r="H97" s="3"/>
+      <c r="H97" s="3" t="s">
+        <v>235</v>
+      </c>
       <c r="I97" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J97" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="H98" s="3"/>
+      <c r="I98" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" s="3" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="99" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="100" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="101" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4106,6 +4133,7 @@
     <row r="1033" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1034" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1035" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1036" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0" footer="0"/>

</xml_diff>